<commit_message>
Refine data layout and EIS visualizations
</commit_message>
<xml_diff>
--- a/results/tables/polarization_curve_points.xlsx
+++ b/results/tables/polarization_curve_points.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -550,7 +550,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -594,7 +594,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -638,7 +638,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -682,7 +682,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -770,7 +770,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -814,7 +814,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -902,7 +902,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -990,7 +990,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E14" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2134,7 +2134,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E48" t="n">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E63" t="n">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E64" t="n">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E65" t="n">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -3366,7 +3366,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E68" t="n">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E69" t="n">
@@ -3498,7 +3498,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -3586,7 +3586,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -3806,7 +3806,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -4026,7 +4026,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_300Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E84" t="n">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E86" t="n">
@@ -4246,7 +4246,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E87" t="n">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -4378,7 +4378,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -4422,7 +4422,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -4598,7 +4598,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E95" t="n">
@@ -4642,7 +4642,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E96" t="n">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E97" t="n">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -4774,7 +4774,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E99" t="n">
@@ -4818,7 +4818,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E101" t="n">
@@ -4906,7 +4906,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E105" t="n">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -5170,7 +5170,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E109" t="n">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E110" t="n">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E111" t="n">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E112" t="n">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -5566,7 +5566,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E117" t="n">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E118" t="n">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E119" t="n">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E120" t="n">
@@ -5742,7 +5742,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_528Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E124" t="n">
@@ -5918,7 +5918,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E125" t="n">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -6050,7 +6050,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -6138,7 +6138,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E130" t="n">
@@ -6182,7 +6182,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -6270,7 +6270,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E134" t="n">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -6446,7 +6446,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E139" t="n">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -6622,7 +6622,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E142" t="n">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -6754,7 +6754,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E144" t="n">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E145" t="n">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E147" t="n">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E148" t="n">
@@ -6974,7 +6974,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E149" t="n">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -7062,7 +7062,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E151" t="n">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E153" t="n">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -7282,7 +7282,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -7326,7 +7326,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E157" t="n">
@@ -7370,7 +7370,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -7414,7 +7414,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -7502,7 +7502,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -7546,7 +7546,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E162" t="n">
@@ -7590,7 +7590,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E163" t="n">
@@ -7634,7 +7634,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -7678,7 +7678,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
+          <t>data\Stack1\PolCurves\RealAgeing_PC_58Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -7722,7 +7722,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -7766,7 +7766,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E167" t="n">
@@ -7810,7 +7810,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -7854,7 +7854,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E169" t="n">
@@ -7898,7 +7898,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E170" t="n">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E172" t="n">
@@ -8030,7 +8030,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E173" t="n">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E175" t="n">
@@ -8162,7 +8162,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E176" t="n">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E177" t="n">
@@ -8250,7 +8250,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -8338,7 +8338,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E180" t="n">
@@ -8382,7 +8382,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E181" t="n">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E182" t="n">
@@ -8470,7 +8470,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E183" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E184" t="n">
@@ -8558,7 +8558,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E185" t="n">
@@ -8602,7 +8602,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E186" t="n">
@@ -8646,7 +8646,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -8690,7 +8690,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -8734,7 +8734,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -8778,7 +8778,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E190" t="n">
@@ -8822,7 +8822,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -8866,7 +8866,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -8910,7 +8910,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E193" t="n">
@@ -8954,7 +8954,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E194" t="n">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E195" t="n">
@@ -9042,7 +9042,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E196" t="n">
@@ -9086,7 +9086,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E197" t="n">
@@ -9130,7 +9130,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E198" t="n">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E199" t="n">
@@ -9218,7 +9218,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -9262,7 +9262,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -9306,7 +9306,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -9350,7 +9350,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -9394,7 +9394,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E204" t="n">
@@ -9438,7 +9438,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E205" t="n">
@@ -9482,7 +9482,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_0_BreakIn_1.xlsx</t>
         </is>
       </c>
       <c r="E206" t="n">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E207" t="n">
@@ -9570,7 +9570,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E208" t="n">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E209" t="n">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E210" t="n">
@@ -9702,7 +9702,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E211" t="n">
@@ -9746,7 +9746,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E212" t="n">
@@ -9790,7 +9790,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E213" t="n">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E214" t="n">
@@ -9878,7 +9878,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E215" t="n">
@@ -9922,7 +9922,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E216" t="n">
@@ -9966,7 +9966,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E217" t="n">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E218" t="n">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E219" t="n">
@@ -10098,7 +10098,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E220" t="n">
@@ -10142,7 +10142,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E221" t="n">
@@ -10186,7 +10186,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E222" t="n">
@@ -10230,7 +10230,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E223" t="n">
@@ -10274,7 +10274,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E224" t="n">
@@ -10318,7 +10318,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E225" t="n">
@@ -10362,7 +10362,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E226" t="n">
@@ -10406,7 +10406,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E227" t="n">
@@ -10450,7 +10450,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E228" t="n">
@@ -10494,7 +10494,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E229" t="n">
@@ -10538,7 +10538,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E230" t="n">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E231" t="n">
@@ -10626,7 +10626,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E232" t="n">
@@ -10670,7 +10670,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E233" t="n">
@@ -10714,7 +10714,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E234" t="n">
@@ -10758,7 +10758,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E235" t="n">
@@ -10802,7 +10802,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E236" t="n">
@@ -10846,7 +10846,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E237" t="n">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E238" t="n">
@@ -10934,7 +10934,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E239" t="n">
@@ -10978,7 +10978,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E240" t="n">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E241" t="n">
@@ -11066,7 +11066,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E242" t="n">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E243" t="n">
@@ -11154,7 +11154,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E244" t="n">
@@ -11198,7 +11198,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E245" t="n">
@@ -11242,7 +11242,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E246" t="n">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_120Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E247" t="n">
@@ -11330,7 +11330,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E248" t="n">
@@ -11374,7 +11374,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E249" t="n">
@@ -11418,7 +11418,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E250" t="n">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E251" t="n">
@@ -11506,7 +11506,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E252" t="n">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E253" t="n">
@@ -11594,7 +11594,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E254" t="n">
@@ -11638,7 +11638,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E255" t="n">
@@ -11682,7 +11682,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E256" t="n">
@@ -11726,7 +11726,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E257" t="n">
@@ -11770,7 +11770,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E258" t="n">
@@ -11814,7 +11814,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E259" t="n">
@@ -11858,7 +11858,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E260" t="n">
@@ -11902,7 +11902,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E261" t="n">
@@ -11946,7 +11946,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E262" t="n">
@@ -11990,7 +11990,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E263" t="n">
@@ -12034,7 +12034,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E264" t="n">
@@ -12078,7 +12078,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E265" t="n">
@@ -12122,7 +12122,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E266" t="n">
@@ -12166,7 +12166,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E267" t="n">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E268" t="n">
@@ -12254,7 +12254,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E269" t="n">
@@ -12298,7 +12298,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E270" t="n">
@@ -12342,7 +12342,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E271" t="n">
@@ -12386,7 +12386,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E272" t="n">
@@ -12430,7 +12430,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E273" t="n">
@@ -12474,7 +12474,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E274" t="n">
@@ -12518,7 +12518,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E275" t="n">
@@ -12562,7 +12562,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E276" t="n">
@@ -12606,7 +12606,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E277" t="n">
@@ -12650,7 +12650,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E278" t="n">
@@ -12694,7 +12694,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E279" t="n">
@@ -12738,7 +12738,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E280" t="n">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E281" t="n">
@@ -12826,7 +12826,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E282" t="n">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E283" t="n">
@@ -12914,7 +12914,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E284" t="n">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E285" t="n">
@@ -13002,7 +13002,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E286" t="n">
@@ -13046,7 +13046,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E287" t="n">
@@ -13090,7 +13090,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>data\Realistic accelerated stress tests for PEM fuel cells Test procedure development based on standardized automotive driving cycles\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
+          <t>data\Stack2\PolCurves\RealAgeing_PC_449Cycles_1.xlsx</t>
         </is>
       </c>
       <c r="E288" t="n">

</xml_diff>